<commit_message>
modele logique + spec techniques c8f225e5fada8d63eebf168ef7e03e535fec6f62
</commit_message>
<xml_diff>
--- a/spec-tech/ig/CodeSystem-pdlgc-repo-type-cs.xlsx
+++ b/spec-tech/ig/CodeSystem-pdlgc-repo-type-cs.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-03T08:42:19+00:00</t>
+    <t>2026-07-09T18:12:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -141,7 +141,7 @@
     <t>TRANSVERSE</t>
   </si>
   <si>
-    <t>Répertoire stockant les données transverses associées à un praticient ou une structure</t>
+    <t>Répertoire stockant les données transverses associées à un praticien ou une structure</t>
   </si>
 </sst>
 </file>

</xml_diff>